<commit_message>
WKBK: regenerate all 188 workbooks clean (remove stale files)
Binned all 238 stale xlsx files (multiple dated versions, old naming
conventions) and regenerated from all 188 generators fresh. Each
WKBK folder now contains exactly 1 current workbook per generator.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/isms-core-framework/A.5-organisational-controls/isms-a.5.31-legal-statutory-regulatory-contractual-requirements/WKBK/ISMS-IMP-A.5.31.1_Regulatory_Inventory_20260301.xlsx
+++ b/isms-core-framework/A.5-organisational-controls/isms-a.5.31-legal-statutory-regulatory-contractual-requirements/WKBK/ISMS-IMP-A.5.31.1_Regulatory_Inventory_20260301.xlsx
@@ -1156,7 +1156,7 @@
         </is>
       </c>
       <c r="P3" s="14" t="n">
-        <v>46082.50844222181</v>
+        <v>46082.74821694789</v>
       </c>
     </row>
     <row r="4">
@@ -1235,7 +1235,7 @@
         </is>
       </c>
       <c r="P4" s="14" t="n">
-        <v>46082.50844222181</v>
+        <v>46082.74821694789</v>
       </c>
     </row>
     <row r="5">
@@ -1314,7 +1314,7 @@
         </is>
       </c>
       <c r="P5" s="14" t="n">
-        <v>46082.50844222181</v>
+        <v>46082.74821694789</v>
       </c>
     </row>
     <row r="6">
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="P6" s="14" t="n">
-        <v>46082.50844222181</v>
+        <v>46082.74821694789</v>
       </c>
     </row>
     <row r="7">
@@ -1472,7 +1472,7 @@
         </is>
       </c>
       <c r="P7" s="14" t="n">
-        <v>46082.50844222181</v>
+        <v>46082.74821694789</v>
       </c>
     </row>
     <row r="8">
@@ -1551,7 +1551,7 @@
         </is>
       </c>
       <c r="P8" s="14" t="n">
-        <v>46082.50844222181</v>
+        <v>46082.74821694789</v>
       </c>
     </row>
     <row r="9">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="P9" s="14" t="n">
-        <v>46082.50844222181</v>
+        <v>46082.74821694789</v>
       </c>
     </row>
     <row r="10">
@@ -1707,7 +1707,7 @@
         </is>
       </c>
       <c r="P10" s="14" t="n">
-        <v>46082.50844222181</v>
+        <v>46082.74821694789</v>
       </c>
     </row>
   </sheetData>

</xml_diff>